<commit_message>
feat: initialize web admin side application with Next.js and TypeScript
- Create layout and page components for the admin console.
- Implement robots.txt to prevent indexing by crawlers.
- Generate theme CSS from design tokens.
- Configure Next.js with API rewrites and package transpilation.
- Add package.json with scripts for development and build processes.
- Set up PostCSS for Tailwind CSS integration.
- Create script to generate theme CSS from tokens.
- Define TypeScript configuration for the application.
- Add TurboRepo configuration for build tasks.
- Introduce admin-related contracts in the contracts package.
- Extend domain package with permission matrix for staff roles.
- Implement permission matrix logic and tests.
- Update i18n messages for admin roles and system health.
</commit_message>
<xml_diff>
--- a/docs/checklists/checklist-milestone-M0-M6.xlsx
+++ b/docs/checklists/checklist-milestone-M0-M6.xlsx
@@ -969,7 +969,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2968,12 +2967,12 @@
       </c>
       <c r="I11" s="36" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="J11" s="37" t="inlineStr">
         <is>
-          <t>Có /health; thiếu readiness kiểm tra DB và Redis.</t>
+          <t>Có /health; thiếu readiness kiểm tra DB và Redis. Xong 24/09/2026: thêm GET /api/v1/health/ready kiểm PostgreSQL + Redis cache + Redis queue, trả 200 hoặc 503 kèm tên dịch vụ đang hỏng (e2e health.e2e.spec.ts; chạy thật: tắt Redis cache → 503, bật lại → 200).</t>
         </is>
       </c>
       <c r="K11" s="37" t="inlineStr">
@@ -2982,7 +2981,11 @@
         </is>
       </c>
       <c r="L11" s="37" t="n"/>
-      <c r="M11" s="37" t="n"/>
+      <c r="M11" s="37" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="94" customHeight="1">
       <c r="A12" s="36" t="n">
@@ -4674,12 +4677,12 @@
       <c r="H7" s="32" t="inlineStr"/>
       <c r="I7" s="32" t="inlineStr">
         <is>
-          <t>Cần chốt</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="J7" s="35" t="inlineStr">
         <is>
-          <t>Hạn 21/09; chặn E2-S7.</t>
+          <t>Hạn 21/09; chặn E2-S7. Chốt 24/09/2026: giữ tên code TrustLevelGuard/@MinTrustLevel; guard mới là RolesGuard/@Roles, thứ tự JwtAuthGuard → RolesGuard → TrustLevelGuard (D-07: role trước trust). Kế hoạch và nghiệm thu: .agent/specs/_changes/rbac-admin-shell/.</t>
         </is>
       </c>
       <c r="K7" s="35" t="inlineStr">
@@ -4688,7 +4691,11 @@
         </is>
       </c>
       <c r="L7" s="35" t="n"/>
-      <c r="M7" s="35" t="n"/>
+      <c r="M7" s="35" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="32" t="n">
@@ -4764,12 +4771,12 @@
       <c r="H9" s="32" t="inlineStr"/>
       <c r="I9" s="32" t="inlineStr">
         <is>
-          <t>Cần chốt</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="J9" s="35" t="inlineStr">
         <is>
-          <t>Hạn 21/09.</t>
+          <t>Hạn 21/09. Chốt 24/09/2026: packages/domain/src/permission-matrix.ts (STAFF_ROLES, SYSTEM_HEALTH_ROLES, PERMISSION_MATRIX), dùng chung cho RolesGuard ở API và menu/chặn route ở web admin; có unit test.</t>
         </is>
       </c>
       <c r="K9" s="35" t="inlineStr">
@@ -4778,7 +4785,11 @@
         </is>
       </c>
       <c r="L9" s="35" t="n"/>
-      <c r="M9" s="35" t="n"/>
+      <c r="M9" s="35" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="49" customHeight="1">
       <c r="A10" s="32" t="n">
@@ -5034,17 +5045,25 @@
       <c r="H15" s="32" t="inlineStr"/>
       <c r="I15" s="32" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="J15" s="35" t="inlineStr"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="J15" s="35" t="inlineStr">
+        <is>
+          <t>Xong 24/09/2026: MailModule gửi qua SMTP (mặc định Mailpit), chặn người nhận theo MAIL_ALLOWED_DOMAINS cho staging, không ghi địa chỉ email vào log (e2e mail.e2e.spec.ts gửi thật và đọc lại từ Mailpit).</t>
+        </is>
+      </c>
       <c r="K15" s="35" t="inlineStr">
         <is>
           <t>Kiểm tra code 18/09/2026</t>
         </is>
       </c>
       <c r="L15" s="35" t="n"/>
-      <c r="M15" s="35" t="n"/>
+      <c r="M15" s="35" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="32" t="n">
@@ -5075,17 +5094,25 @@
       <c r="H16" s="32" t="inlineStr"/>
       <c r="I16" s="32" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="J16" s="35" t="inlineStr"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="J16" s="35" t="inlineStr">
+        <is>
+          <t>Xong 24/09/2026: RedisModule có hai client (cache 6381, queue 6380 cấu hình sẵn cho BullMQ), kết nối lười, log khi mất và khi khôi phục kết nối, đóng sạch khi tắt app (enableShutdownHooks). Hàng đợi BullMQ tạo cùng E7-S1.</t>
+        </is>
+      </c>
       <c r="K16" s="35" t="inlineStr">
         <is>
           <t>Kiểm tra code 18/09/2026</t>
         </is>
       </c>
       <c r="L16" s="35" t="n"/>
-      <c r="M16" s="35" t="n"/>
+      <c r="M16" s="35" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="32" t="n">
@@ -5487,12 +5514,12 @@
       </c>
       <c r="I24" s="36" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="J24" s="37" t="inlineStr">
         <is>
-          <t>Enum 5 role đã đúng; chưa có RolesGuard/@Roles, chỉ có TrustLevelGuard. Tinh gọn: Thuộc danh sách không bao giờ cắt</t>
+          <t>Enum 5 role đã đúng; chưa có RolesGuard/@Roles, chỉ có TrustLevelGuard. Tinh gọn: Thuộc danh sách không bao giờ cắt Xong 24/09/2026: thêm RolesGuard/@Roles và endpoint staff GET /api/v1/admin/system/health; 9 ca e2e admin-system-health.e2e.spec.ts. Kế hoạch và nghiệm thu: .agent/specs/_changes/rbac-admin-shell/.</t>
         </is>
       </c>
       <c r="K24" s="37" t="inlineStr">
@@ -5501,7 +5528,11 @@
         </is>
       </c>
       <c r="L24" s="37" t="n"/>
-      <c r="M24" s="37" t="n"/>
+      <c r="M24" s="37" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="79" customHeight="1">
       <c r="A25" s="36" t="n">
@@ -5948,12 +5979,12 @@
       <c r="H33" s="39" t="inlineStr"/>
       <c r="I33" s="39" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="J33" s="40" t="inlineStr">
         <is>
-          <t>Chưa có RolesGuard.</t>
+          <t>Chưa có RolesGuard. Xong 24/09/2026: member gọi endpoint chỉ dành cho admin → 403 ROLE_NOT_ALLOWED (không 404/500), body không liệt kê role hợp lệ (e2e ca #2). Chưa có endpoint chỉ dành cho moderator nên test dùng endpoint admin.</t>
         </is>
       </c>
       <c r="K33" s="40" t="inlineStr">
@@ -5962,7 +5993,11 @@
         </is>
       </c>
       <c r="L33" s="40" t="n"/>
-      <c r="M33" s="40" t="n"/>
+      <c r="M33" s="40" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="49" customHeight="1">
       <c r="A34" s="39" t="n">
@@ -6312,12 +6347,12 @@
       <c r="H41" s="42" t="inlineStr"/>
       <c r="I41" s="42" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="J41" s="43" t="inlineStr">
         <is>
-          <t>Bằng chứng: Test e2e</t>
+          <t>Bằng chứng: Test e2e Đạt 24/09/2026: curator/moderator/member → 403, admin/super_admin → 200 (e2e ca #2–6).</t>
         </is>
       </c>
       <c r="K41" s="43" t="inlineStr">
@@ -6326,7 +6361,11 @@
         </is>
       </c>
       <c r="L41" s="43" t="n"/>
-      <c r="M41" s="43" t="n"/>
+      <c r="M41" s="43" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="34" customHeight="1">
       <c r="A42" s="42" t="n">
@@ -6688,17 +6727,25 @@
       <c r="H49" s="45" t="inlineStr"/>
       <c r="I49" s="45" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="J49" s="46" t="inlineStr"/>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="J49" s="46" t="inlineStr">
+        <is>
+          <t>Đạt 24/09/2026, cách demo đúng: đổi role trong DB → gọi bằng token cũ vẫn 403 (role nằm trong JWT) → refresh hoặc đăng nhập lại → 200. Dùng cặp member → admin qua GET /api/v1/admin/system/health (e2e ca #7–8).</t>
+        </is>
+      </c>
       <c r="K49" s="46" t="inlineStr">
         <is>
           <t>Doc 08 §6</t>
         </is>
       </c>
       <c r="L49" s="46" t="n"/>
-      <c r="M49" s="46" t="n"/>
+      <c r="M49" s="46" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="49" customHeight="1">
       <c r="A50" s="48" t="n">

</xml_diff>